<commit_message>
看板: 北单26086期xlsx + beidan_cron.sh可执行位
</commit_message>
<xml_diff>
--- a/docs/data/beidan_26086_dashboard.xlsx
+++ b/docs/data/beidan_26086_dashboard.xlsx
@@ -540,7 +540,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽ 北京单场26086期 比赛看板（皇冠历史相同亚盘） — 2026-08-18</t>
+          <t>⚽ 北京单场26086期 比赛看板（皇冠历史相同亚盘） — 2026-08-19</t>
         </is>
       </c>
     </row>
@@ -1264,20 +1264,24 @@
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>55%</t>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>受半球/一球</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1316,20 +1320,24 @@
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>受平手/半球</t>
+        </is>
+      </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1368,20 +1376,24 @@
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>45%</t>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>平手</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1420,20 +1432,24 @@
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>一球</t>
+        </is>
+      </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>
@@ -1472,20 +1488,24 @@
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>45%</t>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>平手</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
     </row>

</xml_diff>